<commit_message>
feat: fixed PO exporting
</commit_message>
<xml_diff>
--- a/public/templates/po-template.xlsx
+++ b/public/templates/po-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BrandonCode\pck-ledger\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A036D9-CFF7-4C36-9412-CC0334C51D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8807C70F-56CA-428A-902E-8653B7C41CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5E6773E2-7222-400F-9EEC-259D3A26E748}"/>
+    <workbookView xWindow="1950" yWindow="600" windowWidth="14400" windowHeight="15600" xr2:uid="{5E6773E2-7222-400F-9EEC-259D3A26E748}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -123,10 +123,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="dd\-mmmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="_-[$Rp-421]* #,##0.00_-;\-[$Rp-421]* #,##0.00_-;_-[$Rp-421]* &quot;-&quot;??_-;_-@"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -213,14 +214,15 @@
       <name val="Trebuchet MS"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -543,7 +545,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -597,15 +599,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -630,45 +623,19 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -678,21 +645,21 @@
     <xf numFmtId="2" fontId="8" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -702,6 +669,47 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1100,25 +1108,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="38"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="40" t="s">
+      <c r="B2" s="55"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
       <c r="F3" s="3"/>
       <c r="G3" s="4" t="s">
         <v>3</v>
@@ -1129,11 +1137,11 @@
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="3"/>
       <c r="G4" s="4" t="s">
         <v>6</v>
@@ -1144,11 +1152,11 @@
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
       <c r="F5" s="3"/>
       <c r="G5" s="7"/>
       <c r="H5" s="3"/>
@@ -1185,19 +1193,19 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="F9" s="43" t="s">
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="F9" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="21"/>
+      <c r="B10" s="60"/>
       <c r="C10" s="9"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -1206,7 +1214,7 @@
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="21"/>
+      <c r="B11" s="60"/>
       <c r="C11" s="9"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -1215,7 +1223,7 @@
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="21"/>
+      <c r="B12" s="60"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -1224,7 +1232,7 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="21"/>
+      <c r="B13" s="60"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="10"/>
@@ -1233,7 +1241,7 @@
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="21"/>
+      <c r="B14" s="60"/>
       <c r="C14" s="13"/>
       <c r="D14" s="3"/>
       <c r="E14" s="10"/>
@@ -1263,11 +1271,11 @@
       <c r="B17" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
       <c r="F17" s="18" t="s">
         <v>15</v>
       </c>
@@ -1279,218 +1287,218 @@
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="21"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
+      <c r="B18" s="61"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
       <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="21"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
+      <c r="B19" s="61"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="21"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="37"/>
+      <c r="B20" s="61"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
       <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="62"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="21"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
+      <c r="B21" s="61"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
       <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="21"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
+      <c r="B22" s="61"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="33"/>
       <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="21"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
+      <c r="B23" s="61"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
       <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="21"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
+      <c r="B24" s="61"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="33"/>
       <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
+      <c r="G24" s="62"/>
+      <c r="H24" s="62"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="21"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
+      <c r="B25" s="61"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="21"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="37"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
+      <c r="G26" s="62"/>
+      <c r="H26" s="62"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="52"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="20"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="62"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="52"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="33"/>
       <c r="F28" s="20"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="20"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="62"/>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
+      <c r="C29" s="45"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="33"/>
       <c r="F29" s="20"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="20"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="62"/>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="52"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="37"/>
+      <c r="C30" s="45"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="33"/>
       <c r="F30" s="20"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="20"/>
+      <c r="G30" s="64"/>
+      <c r="H30" s="62"/>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="59"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="24" t="s">
+      <c r="B31" s="46"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="25" t="s">
+      <c r="G31" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H31" s="26">
+      <c r="H31" s="23">
         <f>H18</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="62"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="28">
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="45"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="46"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="30"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="35"/>
       <c r="F33" s="16"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="29">
+      <c r="G33" s="22"/>
+      <c r="H33" s="26">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="45"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="48"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="51"/>
+      <c r="E34" s="52"/>
       <c r="F34" s="16"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="29">
+      <c r="G34" s="22"/>
+      <c r="H34" s="26">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="49"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="51"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="38"/>
       <c r="F35" s="16"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="29">
+      <c r="G35" s="27"/>
+      <c r="H35" s="26">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="45"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="46"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="35"/>
       <c r="F36" s="16"/>
-      <c r="G36" s="31" t="s">
+      <c r="G36" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="65">
         <f>H31-H35</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="49"/>
-      <c r="C37" s="50"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="51"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="38"/>
       <c r="F37" s="16"/>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="53"/>
-      <c r="C38" s="54"/>
-      <c r="D38" s="54"/>
-      <c r="E38" s="55"/>
+      <c r="B38" s="39"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="41"/>
       <c r="F38" s="16"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
@@ -1508,15 +1516,15 @@
       <c r="F40" s="16"/>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="56" t="s">
+      <c r="B41" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
       <c r="E41" s="2"/>
-      <c r="F41" s="56"/>
-      <c r="G41" s="39"/>
-      <c r="H41" s="39"/>
+      <c r="F41" s="42"/>
+      <c r="G41" s="30"/>
+      <c r="H41" s="30"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
@@ -1559,16 +1567,16 @@
       <c r="H47" s="3"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B48" s="58" t="s">
+      <c r="B48" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="39"/>
-      <c r="F48" s="56" t="s">
+      <c r="C48" s="30"/>
+      <c r="D48" s="30"/>
+      <c r="F48" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="G48" s="39"/>
-      <c r="H48" s="39"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="30"/>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="3"/>
@@ -1580,25 +1588,44 @@
       <c r="H49" s="3"/>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B50" s="41"/>
-      <c r="C50" s="39"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="39"/>
-      <c r="F50" s="39"/>
-      <c r="G50" s="39"/>
-      <c r="H50" s="39"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="30"/>
+      <c r="D50" s="30"/>
+      <c r="E50" s="30"/>
+      <c r="F50" s="30"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="30"/>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B51" s="41"/>
-      <c r="C51" s="39"/>
-      <c r="D51" s="39"/>
-      <c r="E51" s="39"/>
-      <c r="F51" s="39"/>
-      <c r="G51" s="39"/>
-      <c r="H51" s="39"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="30"/>
+      <c r="D51" s="30"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="B51:H51"/>
     <mergeCell ref="C18:E18"/>
@@ -1615,25 +1642,6 @@
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:H9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C6" r:id="rId1" xr:uid="{AEF25034-3454-4087-856B-CA44CE681A7D}"/>

</xml_diff>